<commit_message>
feat: publish latest app updates
</commit_message>
<xml_diff>
--- a/backend/public/CALCULADORA MATERIALES AQUAM.xlsx
+++ b/backend/public/CALCULADORA MATERIALES AQUAM.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Coral - Jorge Cayo" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Citrino - Eugenio Lopez" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Circón - GASTON VILLARUEL" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Aventurina - Vanesa" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="grilla" localSheetId="0" hidden="0" function="0" vbProcedure="0">'CALCULO DE MATERIALES CIRCON'!$P$9:$AB$34</definedName>
@@ -3280,7 +3281,7 @@
           <t>Fecha</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="139" t="inlineStr">
         <is>
           <t>2025-12-20</t>
         </is>
@@ -3292,7 +3293,7 @@
           <t>Cliente</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="139" t="inlineStr">
         <is>
           <t>GASTON VILLARUEL</t>
         </is>
@@ -3304,7 +3305,7 @@
           <t>Domicilio</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="139" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3316,7 +3317,7 @@
           <t>Piscina</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="139" t="inlineStr">
         <is>
           <t>Circón (5.5×2.8 m x 1.3 a 1.4 metros de profundidad)</t>
         </is>
@@ -3328,7 +3329,7 @@
           <t>Volumen</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="139" t="inlineStr">
         <is>
           <t>20.79 m³ / Espejo de agua: 15.40 m²</t>
         </is>
@@ -3376,62 +3377,62 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="139" t="inlineStr">
         <is>
           <t>Longitud de excavación</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="139" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E15" t="n">
+      <c r="E15" s="139" t="n">
         <v>5.8</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="139" t="inlineStr">
         <is>
           <t>Ancho de excavación</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="139" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E16" s="139" t="n">
         <v>3.1</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="139" t="inlineStr">
         <is>
           <t>Profundidad de excavación</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="139" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E17" t="n">
+      <c r="E17" s="139" t="n">
         <v>1.4</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="139" t="inlineStr">
         <is>
           <t>Volumen total de excavación</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="139" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E18" t="n">
+      <c r="E18" s="139" t="n">
         <v>25.172</v>
       </c>
     </row>
@@ -3443,49 +3444,49 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="139" t="inlineStr">
         <is>
           <t>Cemento para la cama</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="139" t="inlineStr">
         <is>
           <t>bolsas de 50kg</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E21" s="139" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="22">
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="139" t="inlineStr">
         <is>
           <t>Arena gruesa</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="139" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="139" t="inlineStr">
         <is>
           <t>1.54</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="139" t="inlineStr">
         <is>
           <t>Mixto para la cama</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="139" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E23" s="139" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3497,62 +3498,62 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="139" t="inlineStr">
         <is>
           <t>Cemento para vereda</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="139" t="inlineStr">
         <is>
           <t>bolsas de 50kg</t>
         </is>
       </c>
-      <c r="E26" t="n">
+      <c r="E26" s="139" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="139" t="inlineStr">
         <is>
           <t>Arena para vereda</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="139" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="139" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="28">
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="139" t="inlineStr">
         <is>
           <t>Piedra para vereda</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="139" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E28" t="n">
+      <c r="E28" s="139" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="29">
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="139" t="inlineStr">
         <is>
           <t>Malla sima</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="139" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E29" t="n">
+      <c r="E29" s="139" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3564,7 +3565,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="139" t="inlineStr">
         <is>
           <t>Sin items de plomería especificados</t>
         </is>
@@ -3578,64 +3579,64 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="139" t="inlineStr">
         <is>
           <t>Bomba</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="139" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E35" t="n">
+      <c r="E35" s="139" t="n">
         <v>1</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="139" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="139" t="inlineStr">
         <is>
           <t>Filtro</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="139" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E36" t="n">
+      <c r="E36" s="139" t="n">
         <v>1</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="139" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="139" t="inlineStr">
         <is>
           <t>Consumo total</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="139" t="inlineStr">
         <is>
           <t>550 W</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="139" t="inlineStr">
         <is>
           <t>Amperaje</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="139" t="inlineStr">
         <is>
           <t>2.5 A</t>
         </is>
@@ -3649,41 +3650,41 @@
       </c>
     </row>
     <row r="41">
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="139" t="inlineStr">
         <is>
           <t>TDH Total (Altura Dinámica Total)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="139" t="inlineStr">
         <is>
           <t>14.16 m</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="139" t="inlineStr">
         <is>
           <t>Altura que debe vencer la bomba</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="139" t="inlineStr">
         <is>
           <t>Pérdida por fricción (succión)</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="139" t="inlineStr">
         <is>
           <t>0.04 m</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="139" t="inlineStr">
         <is>
           <t>Pérdida por fricción (retorno)</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="139" t="inlineStr">
         <is>
           <t>0.11 m</t>
         </is>
@@ -3695,31 +3696,31 @@
           <t>Pérdida por fricción total</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="139" t="inlineStr">
         <is>
           <t>0.15 m</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="139" t="inlineStr">
         <is>
           <t>Pérdida singular (accesorios succión)</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="139" t="inlineStr">
         <is>
           <t>0.19 m</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="139" t="inlineStr">
         <is>
           <t>Pérdida singular (accesorios retorno)</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="139" t="inlineStr">
         <is>
           <t>0.47 m</t>
         </is>
@@ -3731,7 +3732,7 @@
           <t>Pérdida singular total</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="139" t="inlineStr">
         <is>
           <t>0.66 m</t>
         </is>
@@ -3745,24 +3746,24 @@
       </c>
     </row>
     <row r="49">
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="139" t="inlineStr">
         <is>
           <t xml:space="preserve">  -: 0.44 m/s - ⚠ Fuera de rango</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="139" t="inlineStr">
         <is>
           <t>Rango óptimo: 1.5-2.5 m/s</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="139" t="inlineStr">
         <is>
           <t xml:space="preserve">  -: 0.69 m/s - ⚠ Fuera de rango</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="139" t="inlineStr">
         <is>
           <t>Rango óptimo: 1.5-2.5 m/s</t>
         </is>
@@ -3776,21 +3777,21 @@
       </c>
     </row>
     <row r="52">
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="139" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠ Velocidad muy baja (0.44 m/s). Riesgo de sedimentación. Reducir diámetro o aumentar caudal.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="139" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠ Velocidad muy baja (0.69 m/s). Riesgo de sedimentación. Reducir diámetro o aumentar caudal.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="139" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠ Tu bomba seleccionada (Bomba de filtración principal) no tiene suficiente altura: 7.4 m vs 15.6 m requerido</t>
         </is>
@@ -3804,29 +3805,29 @@
       </c>
     </row>
     <row r="57">
-      <c r="B57" t="inlineStr">
+      <c r="B57" s="139" t="inlineStr">
         <is>
           <t>Potencia instalada total</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="139" t="inlineStr">
         <is>
           <t>746 W</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="139" t="inlineStr">
         <is>
           <t>Potencia de demanda (con simultaneidad)</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="139" t="inlineStr">
         <is>
           <t>746 W</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="139" t="inlineStr">
         <is>
           <t>Considera factor de simultaneidad</t>
         </is>
@@ -3838,75 +3839,75 @@
           <t>Corriente total calculada</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E59" s="139" t="inlineStr">
         <is>
           <t>4.69 A</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="139" t="inlineStr">
         <is>
           <t>Con factor de potencia y eficiencia</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="139" t="inlineStr">
         <is>
           <t>Cable recomendado</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="139" t="inlineStr">
         <is>
           <t>1.5 mm²</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="139" t="inlineStr">
         <is>
           <t>Caída de tensión: 1.57% (máx 3%)</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="139" t="inlineStr">
         <is>
           <t>Capacidad de corriente del cable</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E61" s="139" t="inlineStr">
         <is>
           <t>0.0 A</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="139" t="inlineStr">
         <is>
           <t>Interruptor termomagnético (Breaker)</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="139" t="inlineStr">
         <is>
           <t>0 A</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="139" t="inlineStr">
         <is>
           <t>Curva C recomendada</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="139" t="inlineStr">
         <is>
           <t>Diferencial (RCD)</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="139" t="inlineStr">
         <is>
           <t>0 A / 30 mA</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="139" t="inlineStr">
         <is>
           <t>Obligatorio para piscinas</t>
         </is>
@@ -3947,27 +3948,27 @@
       </c>
     </row>
     <row r="66">
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="139" t="inlineStr">
         <is>
           <t>Bomba de filtrado</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="139" t="inlineStr">
         <is>
           <t>745.7 W</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="139" t="inlineStr">
         <is>
           <t>0.00 A</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E66" s="139" t="inlineStr">
         <is>
           <t>0.85</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F66" s="139" t="inlineStr">
         <is>
           <t>Eficiencia: 85%</t>
         </is>
@@ -3981,41 +3982,41 @@
       </c>
     </row>
     <row r="68">
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="139" t="inlineStr">
         <is>
           <t>Consumo diario</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E68" s="139" t="inlineStr">
         <is>
           <t>5.97 kWh</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="139" t="inlineStr">
         <is>
           <t>Costo mensual estimado</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" s="139" t="inlineStr">
         <is>
           <t>$26.85</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="F69" s="139" t="inlineStr">
         <is>
           <t>8 hrs/día promedio</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="139" t="inlineStr">
         <is>
           <t>Costo anual estimado</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E70" s="139" t="inlineStr">
         <is>
           <t>$326.62</t>
         </is>
@@ -4029,7 +4030,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="B73" t="inlineStr">
+      <c r="B73" s="139" t="inlineStr">
         <is>
           <t>Sin mano de obra especificada</t>
         </is>
@@ -4043,63 +4044,63 @@
       </c>
     </row>
     <row r="76">
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="139" t="inlineStr">
         <is>
           <t>1. Marcado y replanteo del terreno</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="B77" t="inlineStr">
+      <c r="B77" s="139" t="inlineStr">
         <is>
           <t>2. Excavación según dimensiones especificadas</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="B78" t="inlineStr">
+      <c r="B78" s="139" t="inlineStr">
         <is>
           <t>3. Preparación de cama de apoyo</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="B79" t="inlineStr">
+      <c r="B79" s="139" t="inlineStr">
         <is>
           <t>4. Instalación de la piscina</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="B80" t="inlineStr">
+      <c r="B80" s="139" t="inlineStr">
         <is>
           <t>5. Instalación hidráulica (plomería)</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="139" t="inlineStr">
         <is>
           <t>6. Instalación eléctrica y equipos</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="139" t="inlineStr">
         <is>
           <t>7. Relleno y compactación</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="B83" t="inlineStr">
+      <c r="B83" s="139" t="inlineStr">
         <is>
           <t>8. Construcción de vereda perimetral</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="139" t="inlineStr">
         <is>
           <t>9. Pruebas de funcionamiento</t>
         </is>
@@ -4113,35 +4114,35 @@
       </c>
     </row>
     <row r="87">
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="139" t="inlineStr">
         <is>
           <t>• Todos los materiales deben cumplir con normas IRAM vigentes</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="139" t="inlineStr">
         <is>
           <t>• La instalación eléctrica debe ser realizada por electricista matriculado</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="139" t="inlineStr">
         <is>
           <t>• Los equipos deben instalarse en lugar ventilado y protegido</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="B90" t="inlineStr">
+      <c r="B90" s="139" t="inlineStr">
         <is>
           <t>• Realizar prueba de estanqueidad antes del llenado final</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="B91" t="inlineStr">
+      <c r="B91" s="139" t="inlineStr">
         <is>
           <t>• Coordinar con albañil para trabajos de vereda y relleno</t>
         </is>
@@ -4149,6 +4150,2019 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <tabColor rgb="FFFFD700"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:AA55"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="10.16015625" defaultRowHeight="12.8" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="34.53" customWidth="1" style="126" min="1" max="1"/>
+    <col width="12.82" customWidth="1" style="126" min="2" max="2"/>
+    <col width="1.12" customWidth="1" style="127" min="3" max="3"/>
+    <col width="15.75" customWidth="1" style="128" min="4" max="4"/>
+    <col width="12.83" customWidth="1" style="128" min="5" max="5"/>
+    <col width="10.16" customWidth="1" style="128" min="6" max="10"/>
+    <col width="12.9" customWidth="1" style="128" min="11" max="11"/>
+    <col width="10.16" customWidth="1" style="128" min="12" max="14"/>
+    <col width="1.26" customWidth="1" style="129" min="15" max="15"/>
+    <col width="9.470000000000001" customWidth="1" style="128" min="16" max="16"/>
+    <col width="7.21" customWidth="1" style="128" min="17" max="17"/>
+    <col width="10.16" customWidth="1" style="128" min="18" max="19"/>
+    <col width="7.12" customWidth="1" style="128" min="20" max="20"/>
+    <col width="10.16" customWidth="1" style="128" min="21" max="22"/>
+    <col width="8.32" customWidth="1" style="128" min="23" max="23"/>
+    <col width="5.5" customWidth="1" style="128" min="24" max="24"/>
+    <col width="4.59" customWidth="1" style="128" min="25" max="25"/>
+    <col width="10.16" customWidth="1" style="128" min="26" max="27"/>
+    <col width="10.16" customWidth="1" style="128" min="29" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="13.8" customHeight="1" s="130">
+      <c r="A1" s="126" t="inlineStr">
+        <is>
+          <t>LARGO</t>
+        </is>
+      </c>
+      <c r="B1" s="126" t="inlineStr">
+        <is>
+          <t>ANCHO</t>
+        </is>
+      </c>
+      <c r="D1" s="128" t="inlineStr">
+        <is>
+          <t>TIPO 1RA</t>
+        </is>
+      </c>
+      <c r="E1" s="128" t="inlineStr">
+        <is>
+          <t>PANDO</t>
+        </is>
+      </c>
+      <c r="F1" s="128" t="inlineStr">
+        <is>
+          <t>HONDO</t>
+        </is>
+      </c>
+      <c r="G1" s="128" t="inlineStr">
+        <is>
+          <t>ESCALERAS</t>
+        </is>
+      </c>
+      <c r="H1" s="128" t="inlineStr">
+        <is>
+          <t>SKIMMER</t>
+        </is>
+      </c>
+      <c r="I1" s="128" t="inlineStr">
+        <is>
+          <t>IZQUIERDO</t>
+        </is>
+      </c>
+      <c r="J1" s="128" t="inlineStr">
+        <is>
+          <t>DERECHO</t>
+        </is>
+      </c>
+      <c r="K1" s="128" t="inlineStr">
+        <is>
+          <t>TIPO LOSETA</t>
+        </is>
+      </c>
+      <c r="L1" s="128" t="inlineStr">
+        <is>
+          <t>ANCHO_AFUERA</t>
+        </is>
+      </c>
+      <c r="M1" s="128" t="inlineStr">
+        <is>
+          <t>LATERAL</t>
+        </is>
+      </c>
+      <c r="N1" s="128" t="inlineStr">
+        <is>
+          <t>CANALETAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13.8" customHeight="1" s="130">
+      <c r="A2" s="131" t="n">
+        <v>9000</v>
+      </c>
+      <c r="B2" s="131" t="n">
+        <v>4000</v>
+      </c>
+      <c r="D2" s="132" t="inlineStr">
+        <is>
+          <t>terminacion</t>
+        </is>
+      </c>
+      <c r="E2" s="133" t="n">
+        <v>1400</v>
+      </c>
+      <c r="F2" s="133" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G2" s="133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="133" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="133" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="133" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="133" t="inlineStr">
+        <is>
+          <t>TERMINACION</t>
+        </is>
+      </c>
+      <c r="L2" s="133" t="n">
+        <v>480</v>
+      </c>
+      <c r="M2" s="133" t="n">
+        <v>500</v>
+      </c>
+      <c r="N2" s="133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" ht="22.15" customHeight="1" s="130">
+      <c r="D3" s="134" t="inlineStr">
+        <is>
+          <t>↑ solo colocar o TERMINACION o LOMO</t>
+        </is>
+      </c>
+      <c r="K3" s="133" t="inlineStr">
+        <is>
+          <t>TERMINACION L</t>
+        </is>
+      </c>
+      <c r="L3" s="133" t="n">
+        <v>480</v>
+      </c>
+      <c r="M3" s="133" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4" ht="13.8" customHeight="1" s="130">
+      <c r="K4" s="133" t="inlineStr">
+        <is>
+          <t>COMUN</t>
+        </is>
+      </c>
+      <c r="L4" s="133" t="n">
+        <v>500</v>
+      </c>
+      <c r="M4" s="133" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="5" ht="13.8" customHeight="1" s="130">
+      <c r="K5" s="133" t="inlineStr">
+        <is>
+          <t>ESQUINERO_ROBA</t>
+        </is>
+      </c>
+      <c r="L5" s="133" t="n">
+        <v>50</v>
+      </c>
+      <c r="M5" s="133" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" ht="12.8" customHeight="1" s="130">
+      <c r="D6" s="135" t="n"/>
+      <c r="M6" s="128" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" ht="34.75" customHeight="1" s="130">
+      <c r="A7" s="139" t="n"/>
+      <c r="B7" s="139" t="n"/>
+      <c r="C7" s="196" t="n"/>
+      <c r="D7" s="138" t="inlineStr">
+        <is>
+          <t>Ancho 1ra Hilada (mm)</t>
+        </is>
+      </c>
+      <c r="E7" s="138" t="inlineStr">
+        <is>
+          <t>Espesor Contrapiso (mm)</t>
+        </is>
+      </c>
+      <c r="F7" s="138" t="inlineStr">
+        <is>
+          <t>Kg Cemento / m³</t>
+        </is>
+      </c>
+      <c r="G7" s="138" t="inlineStr">
+        <is>
+          <t>m³ Arena / m³</t>
+        </is>
+      </c>
+      <c r="H7" s="138" t="inlineStr">
+        <is>
+          <t>m³ Piedra / m³ (o mixto)</t>
+        </is>
+      </c>
+      <c r="I7" s="138" t="inlineStr">
+        <is>
+          <t>Largo Malla (mm)</t>
+        </is>
+      </c>
+      <c r="J7" s="138" t="inlineStr">
+        <is>
+          <t>Ancho Malla (mm)</t>
+        </is>
+      </c>
+      <c r="K7" s="138" t="inlineStr">
+        <is>
+          <t>Mano de Obra / m² #CHINO#</t>
+        </is>
+      </c>
+      <c r="L7" s="138" t="inlineStr">
+        <is>
+          <t>Adicionales</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="13.8" customHeight="1" s="130">
+      <c r="A8" s="139" t="n"/>
+      <c r="B8" s="139" t="n"/>
+      <c r="C8" s="196" t="n"/>
+      <c r="D8" s="142" t="n">
+        <v>480</v>
+      </c>
+      <c r="E8" s="143" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="143" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="143" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H8" s="143" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I8" s="143" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J8" s="143" t="n">
+        <v>2000</v>
+      </c>
+      <c r="K8" s="144" t="n">
+        <v>45000</v>
+      </c>
+      <c r="L8" s="143" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="128" t="inlineStr">
+        <is>
+          <t>ESCALERA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18.65" customHeight="1" s="130">
+      <c r="A9" s="139" t="n"/>
+      <c r="B9" s="139" t="n"/>
+      <c r="C9" s="196" t="n"/>
+      <c r="D9" s="143" t="n"/>
+      <c r="E9" s="147" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" s="143" t="n">
+        <v>25</v>
+      </c>
+      <c r="G9" s="143" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H9" s="143" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="I9" s="143" t="n"/>
+      <c r="J9" s="143" t="n"/>
+      <c r="K9" s="197">
+        <f>ROUND(   (     ( (A2+(I2+J2)*500+2*$D$8)*(B2+(G2+H2)*500+2*$D$8) - A2*B2 )/1000000   )   * $K$8 * (1+$L$8) ,2)</f>
+        <v/>
+      </c>
+      <c r="L9" s="143" t="n"/>
+      <c r="P9" s="148" t="n"/>
+      <c r="Q9" s="148" t="n"/>
+      <c r="R9" s="148" t="n"/>
+      <c r="S9" s="148" t="n"/>
+      <c r="T9" s="148" t="n"/>
+      <c r="U9" s="148" t="n"/>
+      <c r="V9" s="148" t="n"/>
+      <c r="W9" s="148" t="n"/>
+      <c r="X9" s="148" t="n"/>
+      <c r="Y9" s="148" t="n"/>
+      <c r="Z9" s="198" t="n"/>
+    </row>
+    <row r="10" ht="13.8" customHeight="1" s="130">
+      <c r="A10" s="139" t="n"/>
+      <c r="B10" s="139" t="n"/>
+      <c r="C10" s="196" t="n"/>
+      <c r="D10" s="143" t="n"/>
+      <c r="E10" s="143" t="n">
+        <v>50</v>
+      </c>
+      <c r="F10" s="143" t="n"/>
+      <c r="G10" s="143" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="143">
+        <f>0.6</f>
+        <v/>
+      </c>
+      <c r="I10" s="143" t="n"/>
+      <c r="J10" s="143" t="n"/>
+      <c r="K10" s="143" t="n"/>
+      <c r="L10" s="143" t="n"/>
+      <c r="P10" s="149" t="n"/>
+      <c r="Q10" s="149" t="n"/>
+      <c r="R10" s="150" t="n"/>
+      <c r="S10" s="150" t="n"/>
+      <c r="T10" s="150" t="n"/>
+      <c r="U10" s="150" t="n"/>
+      <c r="V10" s="150" t="n"/>
+      <c r="W10" s="150" t="n"/>
+      <c r="X10" s="150" t="n"/>
+      <c r="Y10" s="149" t="n"/>
+      <c r="Z10" s="149" t="n"/>
+    </row>
+    <row r="11" ht="13.8" customHeight="1" s="130">
+      <c r="A11" s="139" t="n"/>
+      <c r="B11" s="139" t="n"/>
+      <c r="C11" s="196" t="n"/>
+      <c r="D11" s="153" t="n"/>
+      <c r="E11" s="153" t="n"/>
+      <c r="P11" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q11" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R11" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S11" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T11" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U11" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V11" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W11" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X11" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y11" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z11" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA11" s="128" t="n"/>
+    </row>
+    <row r="12" ht="12.8" customHeight="1" s="130">
+      <c r="A12" s="199" t="inlineStr">
+        <is>
+          <t>Jesús Olguin</t>
+        </is>
+      </c>
+      <c r="B12" s="157" t="n"/>
+      <c r="C12" s="158" t="n"/>
+      <c r="D12" s="200" t="inlineStr">
+        <is>
+          <t>CHINO</t>
+        </is>
+      </c>
+      <c r="E12" s="157" t="n"/>
+      <c r="H12" s="128" t="inlineStr">
+        <is>
+          <t>unidades</t>
+        </is>
+      </c>
+      <c r="I12" s="128" t="inlineStr">
+        <is>
+          <t>M² X UNIDAD</t>
+        </is>
+      </c>
+      <c r="J12" s="128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M² TOTAL </t>
+        </is>
+      </c>
+      <c r="P12" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q12" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R12" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S12" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T12" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U12" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V12" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W12" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X12" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y12" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z12" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA12" s="128" t="n"/>
+    </row>
+    <row r="13" ht="12.8" customHeight="1" s="130">
+      <c r="A13" s="160" t="inlineStr">
+        <is>
+          <t>SUPERFICIE DE LA CAMA</t>
+        </is>
+      </c>
+      <c r="B13" s="161" t="inlineStr">
+        <is>
+          <t>36.0m2</t>
+        </is>
+      </c>
+      <c r="C13" s="201" t="n"/>
+      <c r="D13" s="202" t="inlineStr">
+        <is>
+          <t>PRIMERA HILADA O ANILLO</t>
+        </is>
+      </c>
+      <c r="E13" s="203" t="inlineStr">
+        <is>
+          <t>52 Terminación</t>
+        </is>
+      </c>
+      <c r="G13" s="128" t="inlineStr">
+        <is>
+          <t>losetas comunes</t>
+        </is>
+      </c>
+      <c r="H13" s="128">
+        <f>COUNTIF(grilla,"C")</f>
+        <v/>
+      </c>
+      <c r="I13" s="165" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J13" s="128">
+        <f>COUNTIF(grilla,"C")*0.25</f>
+        <v/>
+      </c>
+      <c r="P13" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q13" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R13" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S13" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T13" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U13" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V13" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W13" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X13" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y13" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z13" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA13" s="128" t="n"/>
+    </row>
+    <row r="14" ht="14.9" customHeight="1" s="130">
+      <c r="A14" s="160" t="inlineStr">
+        <is>
+          <t>VOLUMEN DE LA CAMA M3</t>
+        </is>
+      </c>
+      <c r="B14" s="161" t="inlineStr">
+        <is>
+          <t>5.0m³</t>
+        </is>
+      </c>
+      <c r="C14" s="201" t="n"/>
+      <c r="D14" s="202" t="inlineStr">
+        <is>
+          <t>ESQUINEROS</t>
+        </is>
+      </c>
+      <c r="E14" s="204" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="128" t="inlineStr">
+        <is>
+          <t>esquineros</t>
+        </is>
+      </c>
+      <c r="H14" s="128">
+        <f>IF(COUNTIF(grilla,"E")=0,"-",COUNTIF(grilla,"E"))</f>
+        <v/>
+      </c>
+      <c r="I14" s="165">
+        <f>0.25-0.05</f>
+        <v/>
+      </c>
+      <c r="J14" s="167">
+        <f>COUNTIF(grilla,"E")*(0.4*0.4 - ($M$6/1000)^2)</f>
+        <v/>
+      </c>
+      <c r="P14" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q14" s="205" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R14" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="S14" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="T14" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="U14" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="V14" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="W14" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X14" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y14" s="205" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z14" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA14" s="128" t="n"/>
+    </row>
+    <row r="15" ht="14.9" customHeight="1" s="130">
+      <c r="A15" s="169" t="inlineStr">
+        <is>
+          <t>ARENA M3</t>
+        </is>
+      </c>
+      <c r="B15" s="173" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="206" t="n"/>
+      <c r="D15" s="202" t="inlineStr">
+        <is>
+          <t>LOSETAS COMUNES</t>
+        </is>
+      </c>
+      <c r="E15" s="204" t="n">
+        <v>194</v>
+      </c>
+      <c r="G15" s="128" t="inlineStr">
+        <is>
+          <t>rejillas</t>
+        </is>
+      </c>
+      <c r="H15" s="128" t="inlineStr">
+        <is>
+          <t>rejillas</t>
+        </is>
+      </c>
+      <c r="I15" s="165" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" s="167" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="139" t="n"/>
+      <c r="P15" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q15" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y15" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z15" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA15" s="128" t="n"/>
+    </row>
+    <row r="16" ht="13.8" customHeight="1" s="130">
+      <c r="A16" s="169" t="inlineStr">
+        <is>
+          <t>MIXTO M3</t>
+        </is>
+      </c>
+      <c r="B16" s="173" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="206" t="n"/>
+      <c r="D16" s="207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M2 DE VEREDA COMPLETA </t>
+        </is>
+      </c>
+      <c r="E16" s="208" t="n">
+        <v>58.87</v>
+      </c>
+      <c r="G16" s="128" t="inlineStr">
+        <is>
+          <t>terminacion</t>
+        </is>
+      </c>
+      <c r="H16" s="128">
+        <f>COUNTIF(grilla,"T")</f>
+        <v/>
+      </c>
+      <c r="I16" s="165" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="J16" s="167">
+        <f>COUNTIF(grilla,"T")*0.24</f>
+        <v/>
+      </c>
+      <c r="K16" s="139" t="n"/>
+      <c r="P16" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q16" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y16" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z16" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA16" s="128" t="n"/>
+    </row>
+    <row r="17" ht="13.8" customHeight="1" s="130">
+      <c r="A17" s="169" t="inlineStr">
+        <is>
+          <t>MALLA</t>
+        </is>
+      </c>
+      <c r="B17" s="173" t="n">
+        <v>42</v>
+      </c>
+      <c r="C17" s="206" t="n"/>
+      <c r="D17" s="207" t="inlineStr">
+        <is>
+          <t>M3 CONTRAPISO VEREDA</t>
+        </is>
+      </c>
+      <c r="E17" s="208" t="n">
+        <v>24</v>
+      </c>
+      <c r="G17" s="128" t="inlineStr">
+        <is>
+          <t>lomo ballena</t>
+        </is>
+      </c>
+      <c r="H17" s="128">
+        <f>IF(COUNTIF(grilla,"L")=0,"-",COUNTIF(grilla,"L"))</f>
+        <v/>
+      </c>
+      <c r="I17" s="165" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J17" s="167">
+        <f>COUNTIF(grilla,"L")*0.2</f>
+        <v/>
+      </c>
+      <c r="K17" s="139" t="n"/>
+      <c r="P17" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q17" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y17" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z17" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA17" s="128" t="n"/>
+    </row>
+    <row r="18" ht="28.35" customHeight="1" s="130">
+      <c r="A18" s="169" t="inlineStr">
+        <is>
+          <t>ARENA PARA TAPADO M3</t>
+        </is>
+      </c>
+      <c r="B18" s="173" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C18" s="206" t="n"/>
+      <c r="D18" s="202" t="inlineStr">
+        <is>
+          <t>BOLSAS DE CEMENTO</t>
+        </is>
+      </c>
+      <c r="E18" s="204" t="n">
+        <v>246</v>
+      </c>
+      <c r="G18" s="128" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="J18" s="128">
+        <f>SUM($J$13:$J$17)</f>
+        <v/>
+      </c>
+      <c r="K18" s="139" t="n"/>
+      <c r="P18" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q18" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y18" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z18" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA18" s="128" t="n"/>
+    </row>
+    <row r="19" ht="14.9" customHeight="1" s="130">
+      <c r="A19" s="169" t="inlineStr">
+        <is>
+          <t>CEMENTO</t>
+        </is>
+      </c>
+      <c r="B19" s="177" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="209" t="n"/>
+      <c r="D19" s="202" t="inlineStr">
+        <is>
+          <t>ARENA M3</t>
+        </is>
+      </c>
+      <c r="E19" s="210" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="139" t="n"/>
+      <c r="K19" s="139" t="n"/>
+      <c r="P19" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q19" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y19" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z19" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA19" s="128" t="n"/>
+    </row>
+    <row r="20" ht="12.8" customHeight="1" s="130">
+      <c r="A20" s="169" t="inlineStr">
+        <is>
+          <t>TEE</t>
+        </is>
+      </c>
+      <c r="B20" s="177" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="209" t="n"/>
+      <c r="D20" s="202" t="inlineStr">
+        <is>
+          <t>PIEDRA</t>
+        </is>
+      </c>
+      <c r="E20" s="210" t="n">
+        <v>5</v>
+      </c>
+      <c r="J20" s="139" t="n"/>
+      <c r="K20" s="139" t="n"/>
+      <c r="P20" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q20" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y20" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z20" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA20" s="128" t="n"/>
+    </row>
+    <row r="21" ht="12.8" customHeight="1" s="130">
+      <c r="A21" s="169" t="inlineStr">
+        <is>
+          <t>CODO 90º</t>
+        </is>
+      </c>
+      <c r="B21" s="177" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="209" t="n"/>
+      <c r="D21" s="202" t="inlineStr">
+        <is>
+          <t>MALLA</t>
+        </is>
+      </c>
+      <c r="E21" s="204" t="n">
+        <v>68</v>
+      </c>
+      <c r="J21" s="139" t="n"/>
+      <c r="K21" s="139" t="n"/>
+      <c r="P21" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q21" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y21" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z21" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA21" s="128" t="n"/>
+    </row>
+    <row r="22" ht="12.8" customHeight="1" s="130">
+      <c r="A22" s="169" t="inlineStr">
+        <is>
+          <t>CODO 45º</t>
+        </is>
+      </c>
+      <c r="B22" s="177" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="209" t="n"/>
+      <c r="D22" s="202" t="inlineStr">
+        <is>
+          <t>ALAMBRE #14 x KG</t>
+        </is>
+      </c>
+      <c r="E22" s="204" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="139" t="n"/>
+      <c r="K22" s="139" t="n"/>
+      <c r="P22" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q22" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y22" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z22" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA22" s="128" t="n"/>
+    </row>
+    <row r="23" ht="12.8" customHeight="1" s="130">
+      <c r="A23" s="169" t="inlineStr">
+        <is>
+          <t>UNION SIMPLE</t>
+        </is>
+      </c>
+      <c r="B23" s="177" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="209" t="n"/>
+      <c r="D23" s="202" t="inlineStr">
+        <is>
+          <t>CLAVOS 2,5 PULGADAS KG</t>
+        </is>
+      </c>
+      <c r="E23" s="204" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="139" t="n"/>
+      <c r="K23" s="139" t="n"/>
+      <c r="P23" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q23" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y23" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z23" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA23" s="128" t="n"/>
+    </row>
+    <row r="24" ht="12.8" customHeight="1" s="130">
+      <c r="A24" s="169" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UNION DOBLE </t>
+        </is>
+      </c>
+      <c r="B24" s="177" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="209" t="n"/>
+      <c r="D24" s="211" t="inlineStr">
+        <is>
+          <t>BOLSAS DE KLAUKOL</t>
+        </is>
+      </c>
+      <c r="E24" s="212" t="n">
+        <v>295</v>
+      </c>
+      <c r="J24" s="139" t="n"/>
+      <c r="K24" s="139" t="n"/>
+      <c r="P24" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q24" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="R24" s="213" t="n"/>
+      <c r="S24" s="128" t="n"/>
+      <c r="T24" s="128" t="n"/>
+      <c r="U24" s="128" t="n"/>
+      <c r="V24" s="128" t="n"/>
+      <c r="W24" s="128" t="n"/>
+      <c r="X24" s="214" t="n"/>
+      <c r="Y24" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z24" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA24" s="128" t="n"/>
+    </row>
+    <row r="25" ht="12.8" customHeight="1" s="130">
+      <c r="A25" s="169" t="inlineStr">
+        <is>
+          <t>LLAVE ESFERICA</t>
+        </is>
+      </c>
+      <c r="B25" s="177" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="209" t="n"/>
+      <c r="D25" s="202" t="n"/>
+      <c r="E25" s="204" t="n"/>
+      <c r="J25" s="139" t="n"/>
+      <c r="K25" s="139" t="n"/>
+      <c r="P25" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q25" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="R25" s="213" t="n"/>
+      <c r="S25" s="128" t="n"/>
+      <c r="T25" s="128" t="n"/>
+      <c r="U25" s="128" t="n"/>
+      <c r="V25" s="128" t="n"/>
+      <c r="W25" s="128" t="n"/>
+      <c r="X25" s="214" t="n"/>
+      <c r="Y25" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z25" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA25" s="128" t="n"/>
+    </row>
+    <row r="26" ht="9.300000000000001" customHeight="1" s="130">
+      <c r="A26" s="169" t="inlineStr">
+        <is>
+          <t>CAÑO 50MM</t>
+        </is>
+      </c>
+      <c r="B26" s="177" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" s="209" t="n"/>
+      <c r="D26" s="202" t="inlineStr">
+        <is>
+          <t>m² de primer anillo perimetral</t>
+        </is>
+      </c>
+      <c r="E26" s="210" t="n">
+        <v>58.87</v>
+      </c>
+      <c r="J26" s="139" t="n"/>
+      <c r="K26" s="139" t="n"/>
+      <c r="L26" s="139" t="n"/>
+      <c r="P26" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q26" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="R26" s="139" t="n"/>
+      <c r="S26" s="139" t="n"/>
+      <c r="T26" s="139" t="n"/>
+      <c r="U26" s="139" t="n"/>
+      <c r="V26" s="139" t="n"/>
+      <c r="W26" s="139" t="n"/>
+      <c r="X26" s="139" t="n"/>
+      <c r="Y26" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z26" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA26" s="128" t="n"/>
+    </row>
+    <row r="27" ht="16.9" customHeight="1" s="130">
+      <c r="A27" s="169" t="inlineStr">
+        <is>
+          <t>PEGAMENTO x 1kg</t>
+        </is>
+      </c>
+      <c r="B27" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="209" t="n"/>
+      <c r="D27" s="202" t="inlineStr">
+        <is>
+          <t>MANO DE OBRA CHINO (BASE)</t>
+        </is>
+      </c>
+      <c r="E27" s="215" t="n">
+        <v>2649150</v>
+      </c>
+      <c r="J27" s="139" t="n"/>
+      <c r="K27" s="139" t="n"/>
+      <c r="L27" s="139" t="n"/>
+      <c r="P27" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q27" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="R27" s="139" t="n"/>
+      <c r="S27" s="139" t="n"/>
+      <c r="T27" s="139" t="n"/>
+      <c r="U27" s="139" t="n"/>
+      <c r="V27" s="139" t="n"/>
+      <c r="W27" s="139" t="n"/>
+      <c r="X27" s="139" t="n"/>
+      <c r="Y27" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z27" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA27" s="128" t="n"/>
+    </row>
+    <row r="28" ht="12.8" customHeight="1" s="130">
+      <c r="A28" s="169" t="inlineStr">
+        <is>
+          <t>GEOTEXTIL O GEOMEMBRANA 400MICRONES X METRO</t>
+        </is>
+      </c>
+      <c r="B28" s="177" t="n">
+        <v>36</v>
+      </c>
+      <c r="C28" s="209" t="n"/>
+      <c r="D28" s="216" t="inlineStr">
+        <is>
+          <t>MANO DE OBRA CHINO (EXTRA)</t>
+        </is>
+      </c>
+      <c r="E28" s="217" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="139" t="n"/>
+      <c r="K28" s="139" t="n"/>
+      <c r="L28" s="139" t="n"/>
+      <c r="P28" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q28" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="R28" s="139" t="n"/>
+      <c r="S28" s="139" t="n"/>
+      <c r="T28" s="139" t="n"/>
+      <c r="U28" s="139" t="n"/>
+      <c r="V28" s="139" t="n"/>
+      <c r="W28" s="139" t="n"/>
+      <c r="X28" s="139" t="n"/>
+      <c r="Y28" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z28" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA28" s="128" t="n"/>
+    </row>
+    <row r="29" ht="12.8" customHeight="1" s="130">
+      <c r="A29" s="169" t="inlineStr">
+        <is>
+          <t>CAÑO AZUL 25MM X METRO</t>
+        </is>
+      </c>
+      <c r="B29" s="177" t="n">
+        <v>30</v>
+      </c>
+      <c r="C29" s="209" t="n"/>
+      <c r="D29" s="139" t="n"/>
+      <c r="J29" s="139" t="n"/>
+      <c r="K29" s="139" t="n"/>
+      <c r="L29" s="139" t="n"/>
+      <c r="P29" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q29" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="R29" s="139" t="n"/>
+      <c r="S29" s="139" t="n"/>
+      <c r="T29" s="139" t="n"/>
+      <c r="U29" s="139" t="n"/>
+      <c r="V29" s="139" t="n"/>
+      <c r="W29" s="139" t="n"/>
+      <c r="X29" s="139" t="n"/>
+      <c r="Y29" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Z29" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA29" s="128" t="n"/>
+    </row>
+    <row r="30" ht="12.8" customHeight="1" s="130">
+      <c r="A30" s="169" t="inlineStr">
+        <is>
+          <t>CONECTORES PARA CORRUGADO DE 25MM</t>
+        </is>
+      </c>
+      <c r="B30" s="177" t="n">
+        <v>20</v>
+      </c>
+      <c r="C30" s="209" t="n"/>
+      <c r="D30" s="139" t="n"/>
+      <c r="J30" s="139" t="n"/>
+      <c r="K30" s="139" t="n"/>
+      <c r="P30" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q30" s="205" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R30" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="S30" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="T30" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="U30" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="V30" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="W30" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="X30" s="150" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="Y30" s="205" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z30" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA30" s="128" t="n"/>
+    </row>
+    <row r="31" ht="12.8" customHeight="1" s="130">
+      <c r="D31" s="139" t="n"/>
+      <c r="J31" s="139" t="n"/>
+      <c r="K31" s="139" t="n"/>
+      <c r="L31" s="139" t="n"/>
+      <c r="M31" s="139" t="n"/>
+      <c r="O31" s="186" t="n"/>
+      <c r="P31" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q31" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R31" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S31" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T31" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U31" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V31" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W31" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X31" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y31" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z31" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA31" s="128" t="n"/>
+    </row>
+    <row r="32" ht="12.8" customHeight="1" s="130">
+      <c r="D32" s="139" t="n"/>
+      <c r="J32" s="139" t="n"/>
+      <c r="K32" s="139" t="n"/>
+      <c r="L32" s="139" t="n"/>
+      <c r="M32" s="139" t="n"/>
+      <c r="O32" s="186" t="n"/>
+      <c r="P32" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q32" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R32" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S32" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T32" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U32" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V32" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W32" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X32" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y32" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z32" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA32" s="128" t="n"/>
+    </row>
+    <row r="33" ht="12.8" customHeight="1" s="130">
+      <c r="A33" s="126" t="inlineStr">
+        <is>
+          <t>Total arena Jesús Olguin ,Vanesa</t>
+        </is>
+      </c>
+      <c r="B33" s="187" t="inlineStr">
+        <is>
+          <t>16.0 m³</t>
+        </is>
+      </c>
+      <c r="C33" s="188" t="n"/>
+      <c r="D33" s="139" t="n"/>
+      <c r="G33" s="139" t="n"/>
+      <c r="H33" s="139" t="n"/>
+      <c r="I33" s="139" t="n"/>
+      <c r="J33" s="139" t="n"/>
+      <c r="K33" s="139" t="n"/>
+      <c r="L33" s="139" t="n"/>
+      <c r="M33" s="139" t="n"/>
+      <c r="N33" s="139" t="n"/>
+      <c r="O33" s="186" t="n"/>
+      <c r="P33" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Q33" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="R33" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S33" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="T33" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="U33" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="V33" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="W33" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X33" s="150" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Y33" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="Z33" s="149" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="AA33" s="128" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="12.8" customHeight="1" s="130">
+      <c r="A34" s="126" t="inlineStr">
+        <is>
+          <t>MIXTO M3</t>
+        </is>
+      </c>
+      <c r="B34" s="189" t="inlineStr">
+        <is>
+          <t>59.0 m³</t>
+        </is>
+      </c>
+      <c r="C34" s="190" t="n"/>
+      <c r="D34" s="139" t="n"/>
+      <c r="J34" s="139" t="n"/>
+      <c r="K34" s="139" t="n"/>
+      <c r="L34" s="139" t="n"/>
+      <c r="M34" s="139" t="n"/>
+      <c r="N34" s="139" t="n"/>
+      <c r="O34" s="186" t="n"/>
+      <c r="P34" s="149" t="n"/>
+      <c r="Q34" s="149" t="n"/>
+      <c r="R34" s="150" t="n"/>
+      <c r="S34" s="150" t="n"/>
+      <c r="T34" s="150" t="n"/>
+      <c r="U34" s="150" t="n"/>
+      <c r="V34" s="150" t="n"/>
+      <c r="W34" s="150" t="n"/>
+      <c r="X34" s="150" t="n"/>
+      <c r="Y34" s="149" t="n"/>
+      <c r="Z34" s="149" t="n"/>
+    </row>
+    <row r="35" ht="12.8" customHeight="1" s="130">
+      <c r="A35" s="139" t="n"/>
+      <c r="B35" s="139" t="n"/>
+      <c r="C35" s="196" t="n"/>
+      <c r="E35" s="139" t="n"/>
+      <c r="F35" s="139" t="n"/>
+      <c r="G35" s="139" t="n"/>
+      <c r="H35" s="139" t="n"/>
+      <c r="J35" s="139" t="n"/>
+      <c r="K35" s="139" t="n"/>
+      <c r="L35" s="139" t="n"/>
+      <c r="M35" s="139" t="n"/>
+      <c r="N35" s="139" t="n"/>
+      <c r="O35" s="186" t="n"/>
+      <c r="P35" s="139" t="n"/>
+      <c r="Q35" s="139" t="n"/>
+      <c r="R35" s="139" t="n"/>
+      <c r="S35" s="139" t="n"/>
+      <c r="T35" s="139" t="n"/>
+    </row>
+    <row r="36" ht="12.8" customHeight="1" s="130">
+      <c r="A36" s="139" t="n"/>
+      <c r="B36" s="139" t="n"/>
+      <c r="C36" s="196" t="n"/>
+      <c r="E36" s="139" t="n"/>
+      <c r="F36" s="139" t="n"/>
+      <c r="G36" s="139" t="n"/>
+      <c r="H36" s="139" t="n"/>
+      <c r="J36" s="139" t="n"/>
+      <c r="K36" s="139" t="n"/>
+      <c r="L36" s="139" t="n"/>
+      <c r="M36" s="139" t="n"/>
+      <c r="N36" s="139" t="n"/>
+      <c r="O36" s="186" t="n"/>
+      <c r="P36" s="139" t="n"/>
+      <c r="Q36" s="139" t="n"/>
+      <c r="R36" s="139" t="n"/>
+      <c r="S36" s="139" t="n"/>
+      <c r="T36" s="139" t="n"/>
+    </row>
+    <row r="37" ht="12.8" customHeight="1" s="130">
+      <c r="A37" s="139" t="n"/>
+      <c r="B37" s="139" t="n"/>
+      <c r="C37" s="196" t="n"/>
+      <c r="E37" s="139" t="n"/>
+      <c r="F37" s="139" t="n"/>
+      <c r="G37" s="139" t="n"/>
+      <c r="H37" s="139" t="n"/>
+      <c r="J37" s="139" t="n"/>
+      <c r="K37" s="139" t="n"/>
+      <c r="L37" s="139" t="n"/>
+      <c r="M37" s="139" t="n"/>
+      <c r="N37" s="139" t="n"/>
+      <c r="O37" s="186" t="n"/>
+      <c r="P37" s="139" t="n"/>
+      <c r="Q37" s="139" t="n"/>
+      <c r="R37" s="139" t="n"/>
+      <c r="S37" s="139" t="n"/>
+      <c r="T37" s="139" t="n"/>
+    </row>
+    <row r="38" ht="12.8" customHeight="1" s="130">
+      <c r="A38" s="139" t="n"/>
+      <c r="B38" s="139" t="n"/>
+      <c r="C38" s="196" t="n"/>
+      <c r="D38" s="218" t="n"/>
+      <c r="E38" s="139" t="n"/>
+      <c r="F38" s="139" t="n"/>
+      <c r="G38" s="139" t="n"/>
+      <c r="H38" s="139" t="n"/>
+      <c r="J38" s="139" t="n"/>
+      <c r="K38" s="139" t="n"/>
+      <c r="L38" s="139" t="n"/>
+      <c r="M38" s="139" t="n"/>
+      <c r="N38" s="139" t="n"/>
+      <c r="O38" s="186" t="n"/>
+      <c r="P38" s="139" t="n"/>
+      <c r="Q38" s="139" t="n"/>
+      <c r="R38" s="139" t="n"/>
+      <c r="S38" s="139" t="n"/>
+      <c r="T38" s="139" t="n"/>
+    </row>
+    <row r="39" ht="12.8" customHeight="1" s="130">
+      <c r="A39" s="139" t="n"/>
+      <c r="B39" s="139" t="n"/>
+      <c r="C39" s="196" t="n"/>
+      <c r="D39" s="218" t="n"/>
+      <c r="E39" s="139" t="n"/>
+      <c r="F39" s="139" t="n"/>
+      <c r="G39" s="139" t="n"/>
+      <c r="H39" s="139" t="n"/>
+      <c r="J39" s="139" t="n"/>
+      <c r="K39" s="139" t="n"/>
+      <c r="L39" s="139" t="n"/>
+      <c r="M39" s="139" t="n"/>
+      <c r="N39" s="139" t="n"/>
+      <c r="O39" s="186" t="n"/>
+      <c r="P39" s="139" t="n"/>
+      <c r="Q39" s="139" t="n"/>
+      <c r="R39" s="139" t="n"/>
+      <c r="S39" s="139" t="n"/>
+      <c r="T39" s="139" t="n"/>
+    </row>
+    <row r="40" ht="12.8" customHeight="1" s="130">
+      <c r="A40" s="139" t="n"/>
+      <c r="B40" s="139" t="n"/>
+      <c r="C40" s="196" t="n"/>
+      <c r="E40" s="139" t="n"/>
+      <c r="F40" s="139" t="n"/>
+      <c r="G40" s="139" t="n"/>
+      <c r="H40" s="139" t="n"/>
+      <c r="J40" s="139" t="n"/>
+      <c r="K40" s="139" t="n"/>
+      <c r="L40" s="139" t="n"/>
+      <c r="M40" s="139" t="n"/>
+      <c r="N40" s="139" t="n"/>
+      <c r="O40" s="186" t="n"/>
+      <c r="P40" s="139" t="n"/>
+      <c r="Q40" s="139" t="n"/>
+      <c r="R40" s="139" t="n"/>
+      <c r="S40" s="139" t="n"/>
+      <c r="T40" s="139" t="n"/>
+    </row>
+    <row r="41" ht="12.8" customHeight="1" s="130">
+      <c r="A41" s="139" t="n"/>
+      <c r="B41" s="139" t="n"/>
+      <c r="C41" s="196" t="n"/>
+      <c r="E41" s="139" t="n"/>
+      <c r="F41" s="139" t="n"/>
+      <c r="G41" s="139" t="n"/>
+      <c r="H41" s="139" t="n"/>
+      <c r="J41" s="139" t="n"/>
+      <c r="K41" s="139" t="n"/>
+      <c r="L41" s="139" t="n"/>
+      <c r="M41" s="139" t="n"/>
+      <c r="N41" s="139" t="n"/>
+      <c r="O41" s="186" t="n"/>
+      <c r="P41" s="139" t="n"/>
+      <c r="Q41" s="139" t="n"/>
+      <c r="R41" s="139" t="n"/>
+      <c r="S41" s="139" t="n"/>
+      <c r="T41" s="139" t="n"/>
+    </row>
+    <row r="42" ht="12.8" customHeight="1" s="130">
+      <c r="A42" s="139" t="n"/>
+      <c r="B42" s="139" t="n"/>
+      <c r="C42" s="196" t="n"/>
+      <c r="E42" s="139" t="n"/>
+      <c r="F42" s="139" t="n"/>
+      <c r="G42" s="139" t="n"/>
+      <c r="H42" s="139" t="n"/>
+      <c r="J42" s="139" t="n"/>
+      <c r="K42" s="139" t="n"/>
+      <c r="L42" s="139" t="n"/>
+      <c r="M42" s="139" t="n"/>
+      <c r="N42" s="139" t="n"/>
+      <c r="O42" s="186" t="n"/>
+      <c r="P42" s="139" t="n"/>
+      <c r="Q42" s="139" t="n"/>
+      <c r="R42" s="139" t="n"/>
+      <c r="S42" s="139" t="n"/>
+      <c r="T42" s="139" t="n"/>
+    </row>
+    <row r="43" ht="12.8" customHeight="1" s="130">
+      <c r="A43" s="139" t="n"/>
+      <c r="B43" s="139" t="n"/>
+      <c r="C43" s="196" t="n"/>
+      <c r="H43" s="219" t="n"/>
+      <c r="J43" s="139" t="n"/>
+      <c r="K43" s="139" t="n"/>
+      <c r="L43" s="139" t="n"/>
+      <c r="M43" s="139" t="n"/>
+      <c r="N43" s="139" t="n"/>
+      <c r="O43" s="186" t="n"/>
+      <c r="P43" s="139" t="n"/>
+      <c r="Q43" s="139" t="n"/>
+      <c r="R43" s="139" t="n"/>
+      <c r="S43" s="139" t="n"/>
+      <c r="T43" s="139" t="n"/>
+    </row>
+    <row r="44" ht="12.8" customHeight="1" s="130">
+      <c r="A44" s="139" t="n"/>
+      <c r="B44" s="139" t="n"/>
+      <c r="C44" s="196" t="n"/>
+      <c r="J44" s="139" t="n"/>
+      <c r="K44" s="139" t="n"/>
+      <c r="L44" s="139" t="n"/>
+      <c r="M44" s="139" t="n"/>
+      <c r="N44" s="139" t="n"/>
+      <c r="O44" s="186" t="n"/>
+      <c r="P44" s="139" t="n"/>
+      <c r="Q44" s="139" t="n"/>
+      <c r="R44" s="139" t="n"/>
+      <c r="S44" s="139" t="n"/>
+      <c r="T44" s="139" t="n"/>
+    </row>
+    <row r="45" ht="12.8" customHeight="1" s="130">
+      <c r="A45" s="139" t="n"/>
+      <c r="B45" s="139" t="n"/>
+      <c r="C45" s="196" t="n"/>
+      <c r="K45" s="139" t="n"/>
+      <c r="L45" s="139" t="n"/>
+      <c r="M45" s="139" t="n"/>
+      <c r="N45" s="139" t="n"/>
+      <c r="O45" s="186" t="n"/>
+      <c r="P45" s="139" t="n"/>
+      <c r="Q45" s="139" t="n"/>
+      <c r="R45" s="139" t="n"/>
+      <c r="S45" s="139" t="n"/>
+      <c r="T45" s="139" t="n"/>
+    </row>
+    <row r="46" ht="12.8" customHeight="1" s="130">
+      <c r="A46" s="139" t="n"/>
+      <c r="B46" s="139" t="n"/>
+      <c r="C46" s="196" t="n"/>
+      <c r="K46" s="139" t="n"/>
+      <c r="L46" s="139" t="n"/>
+      <c r="M46" s="139" t="n"/>
+      <c r="N46" s="139" t="n"/>
+      <c r="O46" s="186" t="n"/>
+      <c r="P46" s="139" t="n"/>
+      <c r="Q46" s="139" t="n"/>
+      <c r="R46" s="139" t="n"/>
+      <c r="S46" s="139" t="n"/>
+      <c r="T46" s="139" t="n"/>
+    </row>
+    <row r="47" ht="12.8" customHeight="1" s="130">
+      <c r="A47" s="139" t="n"/>
+      <c r="B47" s="139" t="n"/>
+      <c r="C47" s="196" t="n"/>
+      <c r="K47" s="139" t="n"/>
+      <c r="L47" s="139" t="n"/>
+      <c r="M47" s="139" t="n"/>
+      <c r="N47" s="139" t="n"/>
+    </row>
+    <row r="48" ht="12.8" customHeight="1" s="130">
+      <c r="A48" s="139" t="n"/>
+      <c r="B48" s="139" t="n"/>
+      <c r="C48" s="196" t="n"/>
+      <c r="J48" s="139" t="n"/>
+      <c r="K48" s="139" t="n"/>
+      <c r="L48" s="139" t="n"/>
+      <c r="M48" s="139" t="n"/>
+      <c r="N48" s="139" t="n"/>
+    </row>
+    <row r="49" ht="12.8" customHeight="1" s="130">
+      <c r="J49" s="139" t="n"/>
+      <c r="K49" s="139" t="n"/>
+      <c r="L49" s="139" t="n"/>
+      <c r="M49" s="139" t="n"/>
+      <c r="N49" s="139" t="n"/>
+    </row>
+    <row r="50" ht="12.8" customHeight="1" s="130">
+      <c r="J50" s="139" t="n"/>
+      <c r="K50" s="139" t="n"/>
+      <c r="L50" s="139" t="n"/>
+      <c r="M50" s="139" t="n"/>
+    </row>
+    <row r="51" ht="12.8" customHeight="1" s="130">
+      <c r="J51" s="139" t="n"/>
+      <c r="K51" s="139" t="n"/>
+      <c r="L51" s="139" t="n"/>
+      <c r="M51" s="139" t="n"/>
+    </row>
+    <row r="52" ht="12.8" customHeight="1" s="130">
+      <c r="J52" s="139" t="n"/>
+      <c r="K52" s="139" t="n"/>
+      <c r="L52" s="139" t="n"/>
+      <c r="M52" s="139" t="n"/>
+    </row>
+    <row r="53" ht="12.8" customHeight="1" s="130">
+      <c r="J53" s="139" t="n"/>
+      <c r="K53" s="139" t="n"/>
+      <c r="L53" s="139" t="n"/>
+      <c r="M53" s="139" t="n"/>
+    </row>
+    <row r="54" ht="12.8" customHeight="1" s="130">
+      <c r="J54" s="139" t="n"/>
+      <c r="K54" s="139" t="n"/>
+      <c r="L54" s="139" t="n"/>
+      <c r="M54" s="139" t="n"/>
+    </row>
+    <row r="55" ht="12.8" customHeight="1" s="130">
+      <c r="M55" s="220" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A12:B12"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 

</xml_diff>